<commit_message>
update logic to allow for verbose answers
</commit_message>
<xml_diff>
--- a/eval/error_analysis/results/analysis_by_qid.xlsx
+++ b/eval/error_analysis/results/analysis_by_qid.xlsx
@@ -9531,7 +9531,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -9761,7 +9761,7 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -9769,7 +9769,7 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -9793,7 +9793,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -9801,7 +9801,7 @@
         </is>
       </c>
       <c r="R5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -9835,7 +9835,7 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -10229,7 +10229,7 @@
         </is>
       </c>
       <c r="N11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -10245,7 +10245,7 @@
         </is>
       </c>
       <c r="R11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -10385,7 +10385,7 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -10393,7 +10393,7 @@
         </is>
       </c>
       <c r="R13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -10493,7 +10493,7 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -10501,7 +10501,7 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -10509,7 +10509,7 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
@@ -10525,7 +10525,7 @@
         </is>
       </c>
       <c r="N15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -10533,7 +10533,7 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -10541,7 +10541,7 @@
         </is>
       </c>
       <c r="R15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -10689,7 +10689,7 @@
         </is>
       </c>
       <c r="R17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -10797,7 +10797,7 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -10829,7 +10829,7 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -11439,7 +11439,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -11463,7 +11463,7 @@
         </is>
       </c>
       <c r="J28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K28" t="inlineStr">
         <is>
@@ -11643,7 +11643,7 @@
         </is>
       </c>
       <c r="R30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31">
@@ -12383,7 +12383,7 @@
         </is>
       </c>
       <c r="R40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41">
@@ -12409,7 +12409,7 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
@@ -12417,7 +12417,7 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
@@ -12425,7 +12425,7 @@
         </is>
       </c>
       <c r="J41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K41" t="inlineStr">
         <is>
@@ -12449,7 +12449,7 @@
         </is>
       </c>
       <c r="P41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q41" t="inlineStr">
         <is>
@@ -12457,7 +12457,7 @@
         </is>
       </c>
       <c r="R41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42">
@@ -12689,7 +12689,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -12837,7 +12837,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -12861,7 +12861,7 @@
         </is>
       </c>
       <c r="J47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K47" t="inlineStr">
         <is>
@@ -12869,7 +12869,7 @@
         </is>
       </c>
       <c r="L47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M47" t="inlineStr">
         <is>
@@ -13231,7 +13231,7 @@
         </is>
       </c>
       <c r="J52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K52" t="inlineStr">
         <is>
@@ -13255,7 +13255,7 @@
         </is>
       </c>
       <c r="P52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q52" t="inlineStr">
         <is>
@@ -13263,7 +13263,7 @@
         </is>
       </c>
       <c r="R52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53">
@@ -13305,7 +13305,7 @@
         </is>
       </c>
       <c r="J53" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K53" t="inlineStr">
         <is>
@@ -13329,7 +13329,7 @@
         </is>
       </c>
       <c r="P53" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q53" t="inlineStr">
         <is>
@@ -13355,7 +13355,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -13445,7 +13445,7 @@
         </is>
       </c>
       <c r="H55" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I55" t="inlineStr"/>
       <c r="J55" t="n">
@@ -13481,7 +13481,7 @@
         </is>
       </c>
       <c r="R55" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="56">
@@ -13663,7 +13663,7 @@
         </is>
       </c>
       <c r="H58" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I58" t="inlineStr">
         <is>
@@ -13671,7 +13671,7 @@
         </is>
       </c>
       <c r="J58" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K58" t="inlineStr">
         <is>
@@ -13695,7 +13695,7 @@
         </is>
       </c>
       <c r="P58" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q58" t="inlineStr">
         <is>
@@ -13703,7 +13703,7 @@
         </is>
       </c>
       <c r="R58" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="59">
@@ -13819,7 +13819,7 @@
         </is>
       </c>
       <c r="J60" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K60" t="inlineStr">
         <is>
@@ -14313,7 +14313,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -14345,7 +14345,7 @@
         </is>
       </c>
       <c r="L67" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M67" t="inlineStr">
         <is>
@@ -14387,7 +14387,7 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -14543,7 +14543,7 @@
         </is>
       </c>
       <c r="H70" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I70" t="inlineStr">
         <is>
@@ -14551,7 +14551,7 @@
         </is>
       </c>
       <c r="J70" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K70" t="inlineStr">
         <is>
@@ -14575,7 +14575,7 @@
         </is>
       </c>
       <c r="P70" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q70" t="inlineStr">
         <is>
@@ -14583,7 +14583,7 @@
         </is>
       </c>
       <c r="R70" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="71">
@@ -14695,7 +14695,7 @@
         </is>
       </c>
       <c r="J72" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K72" t="inlineStr">
         <is>
@@ -14719,7 +14719,7 @@
         </is>
       </c>
       <c r="P72" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q72" t="inlineStr">
         <is>
@@ -14727,7 +14727,7 @@
         </is>
       </c>
       <c r="R72" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="73">
@@ -14835,7 +14835,7 @@
         </is>
       </c>
       <c r="H74" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I74" t="inlineStr">
         <is>
@@ -14843,7 +14843,7 @@
         </is>
       </c>
       <c r="J74" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K74" t="inlineStr">
         <is>
@@ -14859,7 +14859,7 @@
         </is>
       </c>
       <c r="N74" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O74" t="inlineStr">
         <is>
@@ -14867,7 +14867,7 @@
         </is>
       </c>
       <c r="P74" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q74" t="inlineStr">
         <is>
@@ -14875,7 +14875,7 @@
         </is>
       </c>
       <c r="R74" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="75">
@@ -15933,7 +15933,7 @@
         </is>
       </c>
       <c r="H89" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I89" t="inlineStr">
         <is>
@@ -15965,7 +15965,7 @@
         </is>
       </c>
       <c r="P89" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q89" t="inlineStr">
         <is>
@@ -15991,7 +15991,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -16113,7 +16113,7 @@
         </is>
       </c>
       <c r="P91" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q91" t="inlineStr">
         <is>
@@ -16121,7 +16121,7 @@
         </is>
       </c>
       <c r="R91" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="92">
@@ -16657,7 +16657,7 @@
         </is>
       </c>
       <c r="D99" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -16681,7 +16681,7 @@
         </is>
       </c>
       <c r="J99" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K99" t="inlineStr">
         <is>
@@ -16739,7 +16739,7 @@
         </is>
       </c>
       <c r="F100" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G100" t="inlineStr">
         <is>
@@ -17071,7 +17071,7 @@
         </is>
       </c>
       <c r="P104" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q104" t="inlineStr">
         <is>
@@ -17079,7 +17079,7 @@
         </is>
       </c>
       <c r="R104" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="105">
@@ -17829,7 +17829,7 @@
         </is>
       </c>
       <c r="D115" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -18055,7 +18055,7 @@
         </is>
       </c>
       <c r="F118" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G118" t="inlineStr">
         <is>
@@ -18063,7 +18063,7 @@
         </is>
       </c>
       <c r="H118" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I118" t="inlineStr">
         <is>
@@ -18079,7 +18079,7 @@
         </is>
       </c>
       <c r="L118" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M118" t="inlineStr">
         <is>
@@ -18087,7 +18087,7 @@
         </is>
       </c>
       <c r="N118" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
@@ -18095,7 +18095,7 @@
         </is>
       </c>
       <c r="P118" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q118" t="inlineStr">
         <is>
@@ -18103,7 +18103,7 @@
         </is>
       </c>
       <c r="R118" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="119">
@@ -18269,7 +18269,7 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -19297,7 +19297,7 @@
         </is>
       </c>
       <c r="J14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
@@ -19907,7 +19907,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -19915,7 +19915,7 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="n">
@@ -19927,7 +19927,7 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
@@ -19935,7 +19935,7 @@
         </is>
       </c>
       <c r="L23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M23" t="inlineStr">
         <is>
@@ -20059,7 +20059,7 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -20265,7 +20265,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -20347,7 +20347,7 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -20355,7 +20355,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
@@ -20379,7 +20379,7 @@
         </is>
       </c>
       <c r="N29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
@@ -20387,7 +20387,7 @@
         </is>
       </c>
       <c r="P29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
@@ -20395,7 +20395,7 @@
         </is>
       </c>
       <c r="R29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30">
@@ -20507,7 +20507,7 @@
         </is>
       </c>
       <c r="L31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M31" t="inlineStr">
         <is>
@@ -20619,7 +20619,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -20627,7 +20627,7 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -20651,7 +20651,7 @@
         </is>
       </c>
       <c r="L33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M33" t="inlineStr">
         <is>
@@ -20667,7 +20667,7 @@
         </is>
       </c>
       <c r="P33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
@@ -20825,7 +20825,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -20833,7 +20833,7 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -20857,7 +20857,7 @@
         </is>
       </c>
       <c r="L36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M36" t="inlineStr">
         <is>
@@ -21471,7 +21471,7 @@
         </is>
       </c>
       <c r="F45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -21495,7 +21495,7 @@
         </is>
       </c>
       <c r="L45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M45" t="inlineStr">
         <is>
@@ -21503,7 +21503,7 @@
         </is>
       </c>
       <c r="N45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O45" t="inlineStr">
         <is>
@@ -21519,7 +21519,7 @@
         </is>
       </c>
       <c r="R45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46">
@@ -21603,7 +21603,7 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -21627,7 +21627,7 @@
         </is>
       </c>
       <c r="L47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M47" t="inlineStr">
         <is>
@@ -21669,7 +21669,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -21953,7 +21953,7 @@
         </is>
       </c>
       <c r="F52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -22381,7 +22381,7 @@
         </is>
       </c>
       <c r="L58" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M58" t="inlineStr">
         <is>
@@ -22541,7 +22541,7 @@
         </is>
       </c>
       <c r="R60" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="61">
@@ -22715,7 +22715,7 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
@@ -22863,7 +22863,7 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
@@ -22887,7 +22887,7 @@
         </is>
       </c>
       <c r="L65" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M65" t="inlineStr">
         <is>
@@ -23517,7 +23517,7 @@
         </is>
       </c>
       <c r="J74" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K74" t="inlineStr">
         <is>
@@ -23549,7 +23549,7 @@
         </is>
       </c>
       <c r="R74" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="75">
@@ -23567,7 +23567,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -23575,7 +23575,7 @@
         </is>
       </c>
       <c r="F75" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
@@ -23583,7 +23583,7 @@
         </is>
       </c>
       <c r="H75" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I75" t="inlineStr">
         <is>
@@ -23599,7 +23599,7 @@
         </is>
       </c>
       <c r="L75" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M75" t="inlineStr">
         <is>
@@ -23615,7 +23615,7 @@
         </is>
       </c>
       <c r="P75" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q75" t="inlineStr">
         <is>
@@ -23703,7 +23703,7 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -23711,7 +23711,7 @@
         </is>
       </c>
       <c r="F77" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -23735,7 +23735,7 @@
         </is>
       </c>
       <c r="L77" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M77" t="inlineStr">
         <is>
@@ -23743,7 +23743,7 @@
         </is>
       </c>
       <c r="N77" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O77" t="inlineStr">
         <is>
@@ -23751,7 +23751,7 @@
         </is>
       </c>
       <c r="P77" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q77" t="inlineStr">
         <is>
@@ -23759,7 +23759,7 @@
         </is>
       </c>
       <c r="R77" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="78">
@@ -23785,7 +23785,7 @@
         </is>
       </c>
       <c r="F78" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -23809,7 +23809,7 @@
         </is>
       </c>
       <c r="L78" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M78" t="inlineStr">
         <is>
@@ -24461,7 +24461,7 @@
         </is>
       </c>
       <c r="D88" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -24469,7 +24469,7 @@
         </is>
       </c>
       <c r="F88" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G88" t="inlineStr">
         <is>
@@ -24477,7 +24477,7 @@
         </is>
       </c>
       <c r="H88" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I88" t="inlineStr">
         <is>
@@ -24485,7 +24485,7 @@
         </is>
       </c>
       <c r="J88" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K88" t="inlineStr">
         <is>
@@ -24493,7 +24493,7 @@
         </is>
       </c>
       <c r="L88" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M88" t="inlineStr">
         <is>
@@ -24501,7 +24501,7 @@
         </is>
       </c>
       <c r="N88" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O88" t="inlineStr">
         <is>
@@ -24509,7 +24509,7 @@
         </is>
       </c>
       <c r="P88" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q88" t="inlineStr">
         <is>
@@ -24517,7 +24517,7 @@
         </is>
       </c>
       <c r="R88" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="89">
@@ -24613,7 +24613,7 @@
         </is>
       </c>
       <c r="F90" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G90" t="inlineStr">
         <is>
@@ -24815,7 +24815,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -24823,7 +24823,7 @@
         </is>
       </c>
       <c r="F93" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
@@ -24831,7 +24831,7 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I93" t="inlineStr">
         <is>
@@ -24847,7 +24847,7 @@
         </is>
       </c>
       <c r="L93" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M93" t="inlineStr">
         <is>
@@ -24855,7 +24855,7 @@
         </is>
       </c>
       <c r="N93" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O93" t="inlineStr">
         <is>
@@ -24863,7 +24863,7 @@
         </is>
       </c>
       <c r="P93" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q93" t="inlineStr">
         <is>
@@ -24871,7 +24871,7 @@
         </is>
       </c>
       <c r="R93" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="94">
@@ -25157,7 +25157,7 @@
         </is>
       </c>
       <c r="D98" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -25165,7 +25165,7 @@
         </is>
       </c>
       <c r="F98" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G98" t="inlineStr">
         <is>
@@ -25173,7 +25173,7 @@
         </is>
       </c>
       <c r="H98" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I98" t="inlineStr">
         <is>
@@ -25181,7 +25181,7 @@
         </is>
       </c>
       <c r="J98" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K98" t="inlineStr">
         <is>
@@ -25189,7 +25189,7 @@
         </is>
       </c>
       <c r="L98" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M98" t="inlineStr">
         <is>
@@ -25197,7 +25197,7 @@
         </is>
       </c>
       <c r="N98" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
@@ -25205,7 +25205,7 @@
         </is>
       </c>
       <c r="P98" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q98" t="inlineStr">
         <is>
@@ -25213,7 +25213,7 @@
         </is>
       </c>
       <c r="R98" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="99">
@@ -25353,7 +25353,7 @@
         </is>
       </c>
       <c r="P100" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q100" t="inlineStr">
         <is>
@@ -25651,7 +25651,7 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -25659,7 +25659,7 @@
         </is>
       </c>
       <c r="F105" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G105" t="inlineStr">
         <is>
@@ -25675,7 +25675,7 @@
         </is>
       </c>
       <c r="J105" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K105" t="inlineStr">
         <is>
@@ -26087,7 +26087,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -26095,7 +26095,7 @@
         </is>
       </c>
       <c r="F111" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G111" t="inlineStr">
         <is>
@@ -26135,7 +26135,7 @@
         </is>
       </c>
       <c r="P111" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q111" t="inlineStr">
         <is>
@@ -26161,7 +26161,7 @@
         </is>
       </c>
       <c r="D112" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -26169,7 +26169,7 @@
         </is>
       </c>
       <c r="F112" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G112" t="inlineStr">
         <is>
@@ -26177,7 +26177,7 @@
         </is>
       </c>
       <c r="H112" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I112" t="inlineStr">
         <is>
@@ -26185,7 +26185,7 @@
         </is>
       </c>
       <c r="J112" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K112" t="inlineStr">
         <is>
@@ -26193,7 +26193,7 @@
         </is>
       </c>
       <c r="L112" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M112" t="inlineStr">
         <is>
@@ -26209,7 +26209,7 @@
         </is>
       </c>
       <c r="P112" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q112" t="inlineStr">
         <is>
@@ -26217,7 +26217,7 @@
         </is>
       </c>
       <c r="R112" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="113">
@@ -26243,7 +26243,7 @@
         </is>
       </c>
       <c r="F113" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G113" t="inlineStr">
         <is>
@@ -26585,7 +26585,7 @@
         </is>
       </c>
       <c r="F118" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G118" t="inlineStr">
         <is>
@@ -26593,7 +26593,7 @@
         </is>
       </c>
       <c r="H118" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I118" t="inlineStr">
         <is>

</xml_diff>